<commit_message>
fix phân quyền khách hàng
</commit_message>
<xml_diff>
--- a/hrm/.plans/gop-db/list-page-action-column/quy-tac-mau-button.xlsx
+++ b/hrm/.plans/gop-db/list-page-action-column/quy-tac-mau-button.xlsx
@@ -87,7 +87,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -152,6 +152,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF7F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1ABC9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -321,7 +326,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -379,6 +384,9 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -769,6 +777,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -826,34 +835,34 @@
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Duyệt / Hoàn thành / Kích hoạt</t>
+          <t>Duyệt / Gửi duyệt / Hoàn thành / Kích hoạt</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>primary status="success"</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
+          <t>primary  (KHÔNG kèm status)</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>Duyệt</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>#16A34A / #FFFFFF / #16A34A</t>
+          <t>#1ABC9C / #FFFFFF / #1ABC9C</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Duyệt · Hoàn thành</t>
+          <t>Duyệt · Gửi duyệt · Hoàn thành · Kích hoạt</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Gửi duyệt / Khóa / Cảnh báo</t>
+          <t>Khóa / Cảnh báo</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -863,7 +872,7 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Gửi duyệt</t>
+          <t>Khóa</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -873,7 +882,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Gửi duyệt · Khóa</t>
+          <t>Khóa · Cảnh báo</t>
         </is>
       </c>
     </row>
@@ -1066,6 +1075,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>

</xml_diff>